<commit_message>
Replace the dataset and results
</commit_message>
<xml_diff>
--- a/Results/Generator_Flux.1_Analyser_GPT4.1.xlsx
+++ b/Results/Generator_Flux.1_Analyser_GPT4.1.xlsx
@@ -2,40 +2,31 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="0" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="2">
     <font>
-      <name val="宋体"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="宋体"/>
-      <charset val="134"/>
       <b val="1"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <family val="3"/>
-      <sz val="9"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -55,19 +46,10 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
     </border>
   </borders>
   <cellStyleXfs count="1">
@@ -80,7 +62,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="常规" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -444,7 +426,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:K11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="B1" s="1" t="inlineStr">
@@ -499,9 +481,9 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>ANDY WARHOL</t>
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>Andy Warhol</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -511,7 +493,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -531,7 +513,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -546,7 +528,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>1</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -556,9 +538,9 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>CASPAR DAVID FRIEDRICH</t>
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Camille Corot</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -613,9 +595,9 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>EDGAR DEGAS</t>
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>Edgar Degas</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -670,9 +652,9 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>HANS HOLBEIN THE YOUNGER</t>
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>Hans Holbein the Younger</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -727,9 +709,9 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>JEAN-ANTOINE WATTEAU</t>
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>Jacob Jordaens</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -784,9 +766,9 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>JEAN-BAPTISTE CAMILLE COROT</t>
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>Michelangelo</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -841,9 +823,9 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>JOSEPH-MALLORD WILLIAM TURNER</t>
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>Paul Gauguin</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -898,9 +880,9 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>MICHELANGELO BUONARROTI</t>
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>Salvador Dali</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -955,9 +937,9 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>PAUL GAUGUIN</t>
+      <c r="A10" s="1" t="inlineStr">
+        <is>
+          <t>Vasily Vereshchagin</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1012,9 +994,9 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>WILLIAM HOGARTH</t>
+      <c r="A11" s="1" t="inlineStr">
+        <is>
+          <t>William Turner</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1070,6 +1052,5 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="portrait" paperSize="9"/>
 </worksheet>
 </file>
</xml_diff>